<commit_message>
Add tacho output config (JP2=12V), relay requirements for pump/fan, update ballast resistor status (1.8ohm arrived)
- Tacho: Proto Area 4 pin 17, JP2 jumper selects 5V/12V output, tachoDiv=Half for 4-cyl
- Relay: SSM3K357R MOSFETs drive relay coils only (~150mA), NOT direct pump/fan loads
- Ballast: 1.8 ohm 25W arrived, pending installation (3.3 ohm failed on Mar 1)
- Updated T35 pin 34 in xlsx for tacho output
- TunerStudio restore point from Mar 12
</commit_message>
<xml_diff>
--- a/Speeduino Passat.xlsx
+++ b/Speeduino Passat.xlsx
@@ -624,1806 +624,1638 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="21" min="1" max="1"/>
-    <col width="12" customWidth="1" style="21" min="2" max="2"/>
-    <col width="28" customWidth="1" style="21" min="3" max="3"/>
+    <col width="10" customWidth="1" style="21" min="2" max="2"/>
+    <col width="35" customWidth="1" style="21" min="3" max="3"/>
     <col width="14" customWidth="1" style="21" min="4" max="4"/>
     <col width="12" customWidth="1" style="21" min="5" max="5"/>
-    <col width="10" customWidth="1" style="21" min="6" max="6"/>
+    <col width="6" customWidth="1" style="21" min="6" max="6"/>
     <col width="16" customWidth="1" style="21" min="7" max="7"/>
     <col width="14" customWidth="1" style="21" min="8" max="8"/>
-    <col width="60" customWidth="1" style="21" min="9" max="9"/>
+    <col width="55" customWidth="1" style="21" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>T35 Pin</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="0" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="0" t="inlineStr">
         <is>
           <t>Speeduino Pin</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>Old DB27 Pin</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Wire Gauge</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
         <is>
           <t>Wire Color</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="0" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="0" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>POWER</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Main 12V #1 (ign-switched)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Main 12V (ign-switched)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>16 AWG</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
         <is>
           <t>Vermelho</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="0" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Feeds Speeduino main power</t>
+      <c r="I2" s="0" t="inlineStr">
+        <is>
+          <t>ECU relay -&gt; fuse -&gt; Speeduino power</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>POWER</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Main 12V #2 (ign-switched)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Main GND #1</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>9,10</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>4,16</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>Chassis -&gt; Speeduino GND screw terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>POWER</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Main GND #2</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I4" s="0" t="inlineStr">
+        <is>
+          <t>Second ground wire for heater return path</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>POWER</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Injector 12V rail</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>16 AWG</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>Vermelho/Azul</t>
+        </is>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT NEW</t>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>ECU relay -&gt; fuse -&gt; Injector(s) +12V. Separate from ECU power</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>POWER</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>O2 Heater 12V in</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Cinza</t>
+        </is>
+      </c>
+      <c r="H6" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>Fuel pump relay -&gt; 2A inline fuse -&gt; TinyWB H+12V</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>INJ</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>INJ1 signal</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="H7" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I7" s="0" t="inlineStr">
+        <is>
+          <t>TBI single injector. MPI future: cyl 1+4 semi-seq</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>INJ</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>INJ2 signal</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
+        <is>
+          <t>FUTURE MPI</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>Wire when converting to MPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>INJ</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>INJ3 signal</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t>FUTURE MPI</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>Wire when converting to MPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>INJ</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>INJ4 signal</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="0" t="inlineStr">
+        <is>
+          <t>FUTURE MPI</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>Wire when converting to MPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>IGN</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>IGN1 output</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="0" t="inlineStr">
+        <is>
+          <t>FUTURE IGN</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t>Wire to Bosch Module 124 after VIKA distributor install</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>IAC</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>Stepper 1A</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>Cinza</t>
+        </is>
+      </c>
+      <c r="H12" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I12" s="0" t="inlineStr">
+        <is>
+          <t>DRV8825 B1 coil</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>IAC</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>Stepper 1B</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="H13" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I13" s="0" t="inlineStr">
+        <is>
+          <t>DRV8825 B2 coil</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>IAC</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>Stepper 2A</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="H14" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I14" s="0" t="inlineStr">
+        <is>
+          <t>DRV8825 A2 coil</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>IAC</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Stepper 2B</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>Roxo</t>
+        </is>
+      </c>
+      <c r="H15" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I15" s="0" t="inlineStr">
+        <is>
+          <t>DRV8825 A1 coil</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>SENSOR</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>CLT signal</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="H16" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I16" s="0" t="inlineStr">
+        <is>
+          <t>Coolant NTC sensor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>SENSOR</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>IAT signal</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>Castanho claro</t>
+        </is>
+      </c>
+      <c r="H17" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I17" s="0" t="inlineStr">
+        <is>
+          <t>Inlet air temp NTC sensor</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>SENSOR</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>TPS signal</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G18" s="0" t="inlineStr">
+        <is>
+          <t>Cinza claro</t>
+        </is>
+      </c>
+      <c r="H18" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I18" s="0" t="inlineStr">
+        <is>
+          <t>Throttle position 0-5V</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>SENSOR</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Sensor 5V</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>13,28</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>5,10</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
         <is>
           <t>Vermelho</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H19" s="0" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Redundant power feed</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>POWER</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Main GND #1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>9,10</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>4,16</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>16 AWG</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="I19" s="0" t="inlineStr">
+        <is>
+          <t>Shared 5V ref for TPS + Hall sensor</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>SENSOR</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>Sensor GND (shared CLT+IAT+TPS)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
         <is>
           <t>Preto</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H20" s="0" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ECU power ground</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>POWER</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Main GND #2</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>16 AWG</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="I20" s="0" t="inlineStr">
+        <is>
+          <t>Common ground for all sensors</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>TRIGGER</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Trigger signal (Hall)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="H21" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I21" s="0" t="inlineStr">
+        <is>
+          <t>Hall sensor from distributor</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>TRIGGER</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Trigger 5V</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="H22" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I22" s="0" t="inlineStr">
+        <is>
+          <t>Hall sensor power</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>TRIGGER</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Trigger GND (separate wire)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
         <is>
           <t>Preto</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H23" s="0" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Redundant power ground</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>POWER</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Injector 12V rail</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="I23" s="0" t="inlineStr">
+        <is>
+          <t>Separate from sensor GND for noise isolation</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>LSU</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>LSU IP (Nernst+, JPT 1)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>TinyWB IP</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I24" s="0" t="inlineStr">
+        <is>
+          <t>Sensor signal - NOT power!</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>LSU</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>LSU VM (Virtual GND, JPT 2)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>TinyWB VM</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>16 AWG</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Vermelho/Azul</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="H25" s="0" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Common 12V to injector(s). TBI: 1 inj. MPI: splits to 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>POWER</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>O2 Heater 12V in</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="I25" s="0" t="inlineStr">
+        <is>
+          <t>Sensor reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>LSU</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>LSU H- (Heater return, JPT 3)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>TinyWB H-</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="H26" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I26" s="0" t="inlineStr">
+        <is>
+          <t>High current 1A heater ground return</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>LSU</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>LSU H+ (Heater PWM, JPT 4)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>TinyWB H+</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
         <is>
           <t>Cinza</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H27" s="0" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>From fuel pump relay output to TinyWB H+12V. Fuse 2A</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>INJECTION</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>INJ1 signal</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Azul</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="I27" s="0" t="inlineStr">
+        <is>
+          <t>12V PWM from TinyWB to sensor heater</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>LSU</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>LSU IA (Pump current-, JPT 5)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>TinyWB IA</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>Azul bebe</t>
+        </is>
+      </c>
+      <c r="H28" s="0" t="inlineStr">
         <is>
           <t>CURRENT</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Low-side switch. TBI: single injector. MPI: cyl 1+4 (semi-seq)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>INJECTION</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>INJ2 signal</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="I28" s="0" t="inlineStr">
+        <is>
+          <t>Sensor signal wire</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>LSU</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>LSU UN (Nernst-, JPT 6)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>TinyWB UN</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="H29" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I29" s="0" t="inlineStr">
+        <is>
+          <t>Sensor signal - NOT power!</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>Fuel pump relay drive</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>Laranja</t>
+        </is>
+      </c>
+      <c r="H30" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I30" s="0" t="inlineStr">
+        <is>
+          <t>Low-side switch to relay coil</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>Fan relay drive</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>FUTURE MPI</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>MPI: cyl 2+3 (semi-seq) or cyl 2 (sequential)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>INJECTION</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>INJ3 signal</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="H31" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="I31" s="0" t="inlineStr">
+        <is>
+          <t>Low-side switch to fan relay coil</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>Boost solenoid</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>FUTURE MPI</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>MPI: cyl 3 (sequential only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>INJECTION</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>INJ4 signal</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="H32" s="0" t="inlineStr">
+        <is>
+          <t>FUTURE TURBO</t>
+        </is>
+      </c>
+      <c r="I32" s="0" t="inlineStr">
+        <is>
+          <t>Wastegate/boost control solenoid</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>INPUT</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>Clutch switch</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F33" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G33" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>FUTURE MPI</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>MPI: cyl 4 (sequential only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>IGNITION</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>IGN1 output</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="H33" s="0" t="inlineStr">
+        <is>
+          <t>FUTURE</t>
+        </is>
+      </c>
+      <c r="I33" s="0" t="inlineStr">
+        <is>
+          <t>Launch control + anti-stall</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>SPARE</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>Spare / Flex fuel</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>FUTURE IGN</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>To Bosch Module 124 input. Enable after VIKA distributor install</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>IAC</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Stepper 1A</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Cinza</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>DRV8825 B1 coil</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>IAC</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Stepper 1B</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Verde</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>DRV8825 B2 coil</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>IAC</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Stepper 2A</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Amarelo</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>DRV8825 A2 coil</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>IAC</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Stepper 2B</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Roxo</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>DRV8825 A1 coil</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SENSOR</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CLT signal</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Amarelo</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Coolant temp NTC to Speeduino CLT input</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t>SPARE</t>
+        </is>
+      </c>
+      <c r="I34" s="0" t="inlineStr">
+        <is>
+          <t>Proto area 1 - flex fuel or expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>SPARE</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>Tacho output (optional)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SENSOR</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>IAT signal</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Castanho claro</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Inlet air temp NTC to Speeduino IAT input</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SENSOR</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>TPS signal</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Cinza claro</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Throttle position 0-5V to Speeduino TPS input</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SENSOR</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Sensor 5V</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>13,28</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>5,10</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Vermelho</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Shared 5V ref for TPS + sensors</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>SENSOR</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Sensor GND</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Preto</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Common ground for CLT + IAT + TPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>TRIGGER</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Trigger signal (Hall)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Verde</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Hall sensor from distributor. VR1+/Crank input</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>TRIGGER</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Trigger 5V</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Vermelho</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Hall sensor power (shared with sensor 5V on Speeduino)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>TRIGGER</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Trigger GND</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Preto</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Hall sensor ground (separate wire for noise isolation)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>LSU 4.9</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>LSU IP (Nernst+)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>TinyWB IP</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Vermelho</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>JPT pin 1. Sensor signal wire - NOT power!</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>LSU 4.9</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>LSU VM (Virtual GND)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>TinyWB VM</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>CURRENT (optional)</t>
+        </is>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
+        <is>
+          <t>SPARE</t>
+        </is>
+      </c>
+      <c r="I35" s="0" t="inlineStr">
+        <is>
+          <t>Available for future use</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>SPARE</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>Spare</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Amarelo</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>JPT pin 2. Sensor reference</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>LSU 4.9</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>LSU H- (Heater return)</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>TinyWB H-</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Branco</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>JPT pin 3. High current (~1A) heater ground return</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>LSU 4.9</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>LSU H+ (Heater PWM)</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>TinyWB H+</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
+      <c r="F36" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Cinza</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>JPT pin 4. 12V PWM from TinyWB to sensor heater</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>LSU 4.9</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>LSU IA (Pump current-)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>TinyWB IA</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Azul bebe</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>JPT pin 5. Sensor signal wire</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>LSU 4.9</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>LSU UN (Nernst-)</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>TinyWB UN</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>20 AWG</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Preto</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>JPT pin 6. Sensor signal wire - NOT power!</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Fuel pump relay drive</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Laranja</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Low-side switch to relay coil</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Fan relay drive</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Low-side switch to fan relay coil</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Tacho output</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>FUTURE</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Proto area 4 - dashboard tachometer signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Boost solenoid</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>FUTURE TURBO</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Wastegate/boost control solenoid valve</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>INPUT</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Clutch switch</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>FUTURE</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Proto area 5 - for launch control + anti-stall</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="inlineStr">
+      <c r="H36" s="0" t="inlineStr">
         <is>
           <t>SPARE</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Spare / Flex fuel</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>18 AWG</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>SPARE</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Proto area 1 - flex fuel sensor or future expansion</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38">
-        <f>== PIN COUNT SUMMARY ===</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>POWER</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>6</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Main 12V x2, Main GND x2, INJ 12V, O2 Heater 12V</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>INJECTION</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>4</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>INJ1 (current TBI), INJ2-4 (future MPI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>IGNITION</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>IGN1 (future VIKA distributor)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>IAC</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>4</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Stepper 1A/1B/2A/2B</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>SENSOR</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>5</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>CLT, IAT, TPS, Sensor 5V, Sensor GND</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>TRIGGER</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>3</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Hall signal, 5V, GND</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>LSU 4.9</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>6</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>IP, VM, H-, H+, IA, UN (all go to TinyWB inside box)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>OUTPUT</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>3</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Fuel pump, Fan, Tacho</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>FUTURE</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>2</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Boost solenoid, Clutch switch</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>SPARE</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Flex fuel or expansion</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>35</v>
+      <c r="I36" s="0" t="inlineStr">
+        <is>
+          <t>Available for future use</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>